<commit_message>
feat: adopt conditional residual planning for question 2
</commit_message>
<xml_diff>
--- a/src/data/question2_summary.xlsx
+++ b/src/data/question2_summary.xlsx
@@ -445,10 +445,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>24714266.90635828</v>
+        <v>24999506.88062887</v>
       </c>
     </row>
     <row r="12">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>15306749.50323875</v>
+        <v>15512081.63158399</v>
       </c>
     </row>
     <row r="13">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>417720.3571166667</v>
+        <v>346770.9806671028</v>
       </c>
     </row>
     <row r="14">
@@ -591,76 +591,86 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>1635037.492089842</v>
+        <v>1350104.25137767</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>total_cost_yuan</t>
+          <t>scenario_expected_emergency_cost_yuan</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>16941786.9953286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>charge_kwh</t>
+          <t>total_cost_yuan</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>7345597.458376797</v>
+        <v>16862185.88296166</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>discharge_kwh</t>
+          <t>charge_kwh</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>5949933.941285206</v>
+        <v>7387973.345515737</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>surplus_energy_kwh</t>
+          <t>discharge_kwh</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>5797134.251416666</v>
+        <v>5984258.409867739</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>emergency_event_count</t>
+          <t>surplus_energy_kwh</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>4015</v>
+        <v>6003373.430681319</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>soc_min_kwh</t>
+          <t>emergency_event_count</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>1200</v>
+        <v>3605</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>soc_min_kwh</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>soc_max_kwh</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B22" s="3" t="n">
         <v>10800</v>
       </c>
     </row>
@@ -675,15 +685,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -721,89 +731,23 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>seven_day</t>
+          <t>official</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
         <v>1006.52506740959</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>15306749.50323875</v>
+        <v>15512081.63158399</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1635037.492089842</v>
+        <v>1350104.25137767</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>16941786.9953286</v>
+        <v>16862185.88296166</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>5797134.251416666</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>previous_day</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>1187.219746161477</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>12207408.59600693</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>10610439.03490974</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>22817847.63091667</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>3529878.306142717</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>week_type</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>1218.272847875426</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>16526871.68612934</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>3670339.760871858</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>20197211.4470012</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>8043922.44275</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>similar_day</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>1108.573437550222</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>15045949.33632882</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>3427220.224263383</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>18473169.5605922</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>5856571.509450621</v>
+        <v>6003373.430681319</v>
       </c>
     </row>
   </sheetData>
@@ -822,10 +766,10 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -865,19 +809,19 @@
         <v>45736</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>68901.07202540134</v>
+        <v>68043.32498625325</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>41595.16600271601</v>
+        <v>40984.70806785578</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>933.2520833333333</v>
+        <v>1016.217180952381</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>3326.947920591668</v>
+        <v>3711.921537961907</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44922.11392330768</v>
+        <v>44696.62960581769</v>
       </c>
     </row>
     <row r="3">
@@ -885,10 +829,10 @@
         <v>45829</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>78936.55758337498</v>
+        <v>80546.59310216553</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>48872.5978962647</v>
+        <v>49978.00555913725</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0</v>
@@ -897,7 +841,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>48872.5978962647</v>
+        <v>49978.00555913725</v>
       </c>
     </row>
     <row r="4">
@@ -905,19 +849,19 @@
         <v>45923</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>66519.4579935428</v>
+        <v>68733.33629968361</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>41182.85995311627</v>
+        <v>42547.7209817847</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2447.628633333334</v>
+        <v>1252.618547619046</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>10778.75492755</v>
+        <v>5587.684113396424</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>51961.61488066627</v>
+        <v>48135.40509518113</v>
       </c>
     </row>
     <row r="5">
@@ -925,19 +869,19 @@
         <v>46012</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>95396.9273647575</v>
+        <v>97291.07566218516</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>60876.03708462251</v>
+        <v>62288.82392843439</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1155.364249999999</v>
+        <v>769.9179142857136</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>4122.380459741666</v>
+        <v>2826.937384244046</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>64998.41754436418</v>
+        <v>65115.76131267844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: tighten question 2 validation and reporting
</commit_message>
<xml_diff>
--- a/src/data/question2_summary.xlsx
+++ b/src/data/question2_summary.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="策略汇总" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="方案对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="指定日期" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略汇总" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行配置" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方案对比" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指定日期" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -685,6 +686,154 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>参数</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>forecast_method</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>seven_day</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>planner</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>planning_quantile</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>planning_method</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>conditional_residual</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>residual_candidate_count</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>residual_decay</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>scenario_count</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>scenario_decay</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>execution_strategy</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>fixed_plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>elapsed_seconds</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>4.091192199994111</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>simulated_days</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -755,7 +904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>